<commit_message>
trabajando en la exportacion poa
</commit_message>
<xml_diff>
--- a/assets/video/FORMULARIOSPOA/FORM_MOD_4_Y_5_2026.xlsx
+++ b/assets/video/FORMULARIOSPOA/FORM_MOD_4_Y_5_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp56\htdocs\Siiplas-ci1.5\assets\video\FORMULARIOSPOA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F9A746-B4DA-42B6-8479-1A83B504E269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BC844E-07B8-4704-8AA5-3F6633918E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="543" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="166">
   <si>
     <t>DETALLE</t>
   </si>
@@ -1505,9 +1505,6 @@
     <t>REGIONAL / DEPARTAMENTO:</t>
   </si>
   <si>
-    <t>cite 1</t>
-  </si>
-  <si>
     <t>ADMINISTRACION CENTRAL</t>
   </si>
   <si>
@@ -1517,28 +1514,64 @@
     <t>GERENCIA GENERAL</t>
   </si>
   <si>
-    <t>DPTO. NAL. DE SISTEMAS</t>
-  </si>
-  <si>
-    <t>EN CUMPLIMIENTO A INSTRUCTIVO N° XXX DE FECHA XX/XX/XX</t>
-  </si>
-  <si>
-    <t>VIATICOS</t>
-  </si>
-  <si>
     <t>VIATICO</t>
   </si>
   <si>
     <t>NOVIEMBRE</t>
   </si>
   <si>
-    <t>JEFATURA DNS</t>
-  </si>
-  <si>
-    <t>VIATICOS A SANTA CRUZ</t>
-  </si>
-  <si>
     <t>MARZO</t>
+  </si>
+  <si>
+    <t>DPTO. NAL. DE PLANIFICACION</t>
+  </si>
+  <si>
+    <t>EN CUMPLIMIENTO A INSTRUCTIVO XX SE SOLICITA LA MODIFICACION DE TEMPORALIDAD</t>
+  </si>
+  <si>
+    <t>ACTUALIZACION DEL PLAN ESTRATEGICO INSTITUCIONAL 2026-2030</t>
+  </si>
+  <si>
+    <t>OBJETIVOS ESTRATEGICOS INSTITUCIONALES DEFINIDOS EN EL MARCO DEL PGDEES</t>
+  </si>
+  <si>
+    <t>Nø DE DOCUMENTOS ELABORADOS</t>
+  </si>
+  <si>
+    <t>ABRIL</t>
+  </si>
+  <si>
+    <t>DOCUMENTO PEI ELABORADO Y APROBADO</t>
+  </si>
+  <si>
+    <t>MAYO</t>
+  </si>
+  <si>
+    <t>DNP 1</t>
+  </si>
+  <si>
+    <t>DNP 2</t>
+  </si>
+  <si>
+    <t>EN CUMPLIMIENTO A INSTRUCTIVO N° XXX DE FECHA XX/XX/XX SE SOLICITA LA MODIFICACION E INCLUSION DE REQUERIMIENTO SEGÚN EL SIGUIENTE DETALLE DEL POA ACTUALIZADO</t>
+  </si>
+  <si>
+    <t>VIATICOS ELABORACION DE NORMATIVA</t>
+  </si>
+  <si>
+    <t>VIATICOS A REGIONAL SANTA CRUZ</t>
+  </si>
+  <si>
+    <t>MAYO - NOVIEMBRE</t>
+  </si>
+  <si>
+    <t>DPTO. NAL. PLANIFICACION</t>
+  </si>
+  <si>
+    <t>DOCUMENTO PEI ELABORADO Y APROBADO XX</t>
+  </si>
+  <si>
+    <t>VIATICOS AL INTERIOR DEL PAIS - REGIONAL SANTA CRUZ</t>
   </si>
 </sst>
 </file>
@@ -1548,7 +1581,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="41" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1824,6 +1857,29 @@
     <font>
       <b/>
       <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2118,7 +2174,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="21" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2268,18 +2324,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="34" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2325,116 +2369,134 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="25" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2442,15 +2504,45 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2460,80 +2552,86 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="39" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="40" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="43" fontId="39" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3935,66 +4033,66 @@
     </row>
     <row r="3" spans="2:19" ht="3" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="45"/>
-      <c r="C3" s="100"/>
-      <c r="D3" s="100"/>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="100"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="100"/>
-      <c r="L3" s="100"/>
-      <c r="M3" s="100"/>
-      <c r="N3" s="100"/>
-      <c r="O3" s="100"/>
-      <c r="P3" s="100"/>
-      <c r="Q3" s="100"/>
-      <c r="R3" s="100"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="109"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="109"/>
+      <c r="H3" s="109"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="109"/>
+      <c r="K3" s="109"/>
+      <c r="L3" s="109"/>
+      <c r="M3" s="109"/>
+      <c r="N3" s="109"/>
+      <c r="O3" s="109"/>
+      <c r="P3" s="109"/>
+      <c r="Q3" s="109"/>
+      <c r="R3" s="109"/>
       <c r="S3" s="46"/>
     </row>
     <row r="4" spans="2:19" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="45"/>
-      <c r="C4" s="115" t="s">
+      <c r="C4" s="85" t="s">
         <v>133</v>
       </c>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="115"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="85"/>
+      <c r="I4" s="85"/>
+      <c r="J4" s="85"/>
+      <c r="K4" s="85"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="85"/>
+      <c r="O4" s="85"/>
+      <c r="P4" s="85"/>
+      <c r="Q4" s="85"/>
+      <c r="R4" s="85"/>
       <c r="S4" s="46"/>
     </row>
     <row r="5" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="45"/>
-      <c r="C5" s="114" t="s">
+      <c r="C5" s="84" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="114"/>
-      <c r="E5" s="114"/>
-      <c r="F5" s="114"/>
-      <c r="G5" s="114"/>
-      <c r="H5" s="114"/>
-      <c r="I5" s="114"/>
-      <c r="J5" s="114"/>
-      <c r="K5" s="114"/>
-      <c r="L5" s="114"/>
-      <c r="M5" s="114"/>
-      <c r="N5" s="114"/>
-      <c r="O5" s="114"/>
-      <c r="P5" s="114"/>
-      <c r="Q5" s="114"/>
-      <c r="R5" s="114"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="84"/>
+      <c r="N5" s="84"/>
+      <c r="O5" s="84"/>
+      <c r="P5" s="84"/>
+      <c r="Q5" s="84"/>
+      <c r="R5" s="84"/>
       <c r="S5" s="46"/>
     </row>
     <row r="6" spans="2:19" ht="21" x14ac:dyDescent="0.35">
@@ -4014,9 +4112,11 @@
       <c r="O6" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="117"/>
-      <c r="Q6" s="118"/>
-      <c r="R6" s="119"/>
+      <c r="P6" s="90" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q6" s="91"/>
+      <c r="R6" s="92"/>
       <c r="S6" s="46"/>
     </row>
     <row r="7" spans="2:19" ht="6" customHeight="1" x14ac:dyDescent="0.3">
@@ -4041,15 +4141,15 @@
     </row>
     <row r="8" spans="2:19" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="45"/>
-      <c r="C8" s="121" t="s">
+      <c r="C8" s="94" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="121"/>
-      <c r="E8" s="122">
-        <v>46275</v>
-      </c>
-      <c r="F8" s="123"/>
-      <c r="G8" s="124"/>
+      <c r="D8" s="94"/>
+      <c r="E8" s="95">
+        <v>46091</v>
+      </c>
+      <c r="F8" s="96"/>
+      <c r="G8" s="97"/>
       <c r="H8" s="42"/>
       <c r="I8" s="42"/>
       <c r="J8" s="42"/>
@@ -4082,24 +4182,24 @@
     </row>
     <row r="10" spans="2:19" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="45"/>
-      <c r="C10" s="120" t="s">
+      <c r="C10" s="93" t="s">
         <v>140</v>
       </c>
-      <c r="D10" s="120"/>
-      <c r="E10" s="120"/>
-      <c r="F10" s="120"/>
-      <c r="G10" s="120"/>
-      <c r="H10" s="120"/>
-      <c r="I10" s="120"/>
-      <c r="J10" s="120"/>
-      <c r="K10" s="120"/>
-      <c r="L10" s="120"/>
-      <c r="M10" s="120"/>
-      <c r="N10" s="120"/>
-      <c r="O10" s="120"/>
-      <c r="P10" s="120"/>
-      <c r="Q10" s="120"/>
-      <c r="R10" s="120"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
+      <c r="H10" s="93"/>
+      <c r="I10" s="93"/>
+      <c r="J10" s="93"/>
+      <c r="K10" s="93"/>
+      <c r="L10" s="93"/>
+      <c r="M10" s="93"/>
+      <c r="N10" s="93"/>
+      <c r="O10" s="93"/>
+      <c r="P10" s="93"/>
+      <c r="Q10" s="93"/>
+      <c r="R10" s="93"/>
       <c r="S10" s="46"/>
     </row>
     <row r="11" spans="2:19" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4137,31 +4237,33 @@
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" s="45"/>
-      <c r="C14" s="103" t="s">
+      <c r="C14" s="89" t="s">
         <v>142</v>
       </c>
-      <c r="D14" s="103"/>
-      <c r="E14" s="103"/>
+      <c r="D14" s="89"/>
+      <c r="E14" s="89"/>
       <c r="F14" s="20"/>
-      <c r="G14" s="116"/>
-      <c r="H14" s="116"/>
-      <c r="I14" s="116"/>
-      <c r="J14" s="116"/>
-      <c r="K14" s="116"/>
-      <c r="L14" s="116"/>
-      <c r="M14" s="116"/>
-      <c r="N14" s="116"/>
-      <c r="O14" s="116"/>
-      <c r="P14" s="116"/>
-      <c r="Q14" s="116"/>
-      <c r="R14" s="116"/>
+      <c r="G14" s="88" t="s">
+        <v>143</v>
+      </c>
+      <c r="H14" s="88"/>
+      <c r="I14" s="88"/>
+      <c r="J14" s="88"/>
+      <c r="K14" s="88"/>
+      <c r="L14" s="88"/>
+      <c r="M14" s="88"/>
+      <c r="N14" s="88"/>
+      <c r="O14" s="88"/>
+      <c r="P14" s="88"/>
+      <c r="Q14" s="88"/>
+      <c r="R14" s="88"/>
       <c r="S14" s="46"/>
     </row>
     <row r="15" spans="2:19" ht="3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="45"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="84"/>
-      <c r="E15" s="84"/>
+      <c r="C15" s="80"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="80"/>
       <c r="F15" s="35"/>
       <c r="G15" s="53"/>
       <c r="H15" s="53"/>
@@ -4179,31 +4281,33 @@
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" s="45"/>
-      <c r="C16" s="103" t="s">
+      <c r="C16" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="103"/>
-      <c r="E16" s="103"/>
+      <c r="D16" s="89"/>
+      <c r="E16" s="89"/>
       <c r="F16" s="38"/>
-      <c r="G16" s="116"/>
-      <c r="H16" s="116"/>
-      <c r="I16" s="116"/>
-      <c r="J16" s="116"/>
-      <c r="K16" s="116"/>
-      <c r="L16" s="116"/>
-      <c r="M16" s="116"/>
-      <c r="N16" s="116"/>
-      <c r="O16" s="116"/>
-      <c r="P16" s="116"/>
-      <c r="Q16" s="116"/>
-      <c r="R16" s="116"/>
+      <c r="G16" s="88" t="s">
+        <v>144</v>
+      </c>
+      <c r="H16" s="88"/>
+      <c r="I16" s="88"/>
+      <c r="J16" s="88"/>
+      <c r="K16" s="88"/>
+      <c r="L16" s="88"/>
+      <c r="M16" s="88"/>
+      <c r="N16" s="88"/>
+      <c r="O16" s="88"/>
+      <c r="P16" s="88"/>
+      <c r="Q16" s="88"/>
+      <c r="R16" s="88"/>
       <c r="S16" s="46"/>
     </row>
     <row r="17" spans="2:19" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="45"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="84"/>
+      <c r="C17" s="80"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="80"/>
       <c r="F17" s="35"/>
       <c r="G17" s="53"/>
       <c r="H17" s="53"/>
@@ -4221,31 +4325,33 @@
     </row>
     <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" s="45"/>
-      <c r="C18" s="103" t="s">
+      <c r="C18" s="89" t="s">
         <v>139</v>
       </c>
-      <c r="D18" s="103"/>
-      <c r="E18" s="103"/>
+      <c r="D18" s="89"/>
+      <c r="E18" s="89"/>
       <c r="F18" s="38"/>
-      <c r="G18" s="116"/>
-      <c r="H18" s="116"/>
-      <c r="I18" s="116"/>
-      <c r="J18" s="116"/>
-      <c r="K18" s="116"/>
-      <c r="L18" s="116"/>
-      <c r="M18" s="116"/>
-      <c r="N18" s="116"/>
-      <c r="O18" s="116"/>
-      <c r="P18" s="116"/>
-      <c r="Q18" s="116"/>
-      <c r="R18" s="116"/>
+      <c r="G18" s="88" t="s">
+        <v>145</v>
+      </c>
+      <c r="H18" s="88"/>
+      <c r="I18" s="88"/>
+      <c r="J18" s="88"/>
+      <c r="K18" s="88"/>
+      <c r="L18" s="88"/>
+      <c r="M18" s="88"/>
+      <c r="N18" s="88"/>
+      <c r="O18" s="88"/>
+      <c r="P18" s="88"/>
+      <c r="Q18" s="88"/>
+      <c r="R18" s="88"/>
       <c r="S18" s="46"/>
     </row>
     <row r="19" spans="2:19" ht="3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="45"/>
-      <c r="C19" s="84"/>
-      <c r="D19" s="84"/>
-      <c r="E19" s="84"/>
+      <c r="C19" s="80"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="80"/>
       <c r="F19" s="35"/>
       <c r="G19" s="53"/>
       <c r="H19" s="53"/>
@@ -4263,24 +4369,26 @@
     </row>
     <row r="20" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B20" s="45"/>
-      <c r="C20" s="103" t="s">
+      <c r="C20" s="89" t="s">
         <v>125</v>
       </c>
-      <c r="D20" s="103"/>
-      <c r="E20" s="103"/>
+      <c r="D20" s="89"/>
+      <c r="E20" s="89"/>
       <c r="F20" s="20"/>
-      <c r="G20" s="116"/>
-      <c r="H20" s="116"/>
-      <c r="I20" s="116"/>
-      <c r="J20" s="116"/>
-      <c r="K20" s="116"/>
-      <c r="L20" s="116"/>
-      <c r="M20" s="116"/>
-      <c r="N20" s="116"/>
-      <c r="O20" s="116"/>
-      <c r="P20" s="116"/>
-      <c r="Q20" s="116"/>
-      <c r="R20" s="116"/>
+      <c r="G20" s="88" t="s">
+        <v>149</v>
+      </c>
+      <c r="H20" s="88"/>
+      <c r="I20" s="88"/>
+      <c r="J20" s="88"/>
+      <c r="K20" s="88"/>
+      <c r="L20" s="88"/>
+      <c r="M20" s="88"/>
+      <c r="N20" s="88"/>
+      <c r="O20" s="88"/>
+      <c r="P20" s="88"/>
+      <c r="Q20" s="88"/>
+      <c r="R20" s="88"/>
       <c r="S20" s="46"/>
     </row>
     <row r="21" spans="2:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4302,24 +4410,24 @@
     </row>
     <row r="22" spans="2:19" s="63" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="61"/>
-      <c r="C22" s="90" t="s">
+      <c r="C22" s="98" t="s">
         <v>119</v>
       </c>
-      <c r="D22" s="90"/>
-      <c r="E22" s="90"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="90"/>
-      <c r="H22" s="90"/>
-      <c r="I22" s="90"/>
-      <c r="J22" s="90"/>
-      <c r="K22" s="90"/>
-      <c r="L22" s="90"/>
-      <c r="M22" s="90"/>
-      <c r="N22" s="90"/>
-      <c r="O22" s="90"/>
-      <c r="P22" s="90"/>
-      <c r="Q22" s="90"/>
-      <c r="R22" s="90"/>
+      <c r="D22" s="98"/>
+      <c r="E22" s="98"/>
+      <c r="F22" s="98"/>
+      <c r="G22" s="98"/>
+      <c r="H22" s="98"/>
+      <c r="I22" s="98"/>
+      <c r="J22" s="98"/>
+      <c r="K22" s="98"/>
+      <c r="L22" s="98"/>
+      <c r="M22" s="98"/>
+      <c r="N22" s="98"/>
+      <c r="O22" s="98"/>
+      <c r="P22" s="98"/>
+      <c r="Q22" s="98"/>
+      <c r="R22" s="98"/>
       <c r="S22" s="65"/>
     </row>
     <row r="23" spans="2:19" ht="9" customHeight="1" x14ac:dyDescent="0.25">
@@ -4344,25 +4452,25 @@
     </row>
     <row r="24" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B24" s="45"/>
-      <c r="D24" s="110" t="s">
+      <c r="D24" s="103" t="s">
         <v>108</v>
       </c>
-      <c r="E24" s="111"/>
-      <c r="F24" s="98"/>
-      <c r="G24" s="98"/>
-      <c r="H24" s="109" t="s">
+      <c r="E24" s="104"/>
+      <c r="F24" s="116"/>
+      <c r="G24" s="116"/>
+      <c r="H24" s="102" t="s">
         <v>141</v>
       </c>
-      <c r="I24" s="110"/>
-      <c r="J24" s="110"/>
-      <c r="K24" s="111"/>
-      <c r="L24" s="79"/>
+      <c r="I24" s="103"/>
+      <c r="J24" s="103"/>
+      <c r="K24" s="104"/>
+      <c r="L24" s="75"/>
       <c r="M24" s="57"/>
-      <c r="N24" s="110" t="s">
+      <c r="N24" s="103" t="s">
         <v>109</v>
       </c>
-      <c r="O24" s="111"/>
-      <c r="P24" s="81" t="s">
+      <c r="O24" s="104"/>
+      <c r="P24" s="77" t="s">
         <v>131</v>
       </c>
       <c r="S24" s="46"/>
@@ -4386,66 +4494,68 @@
     </row>
     <row r="26" spans="2:19" s="63" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="61"/>
-      <c r="C26" s="90" t="s">
+      <c r="C26" s="98" t="s">
         <v>104</v>
       </c>
-      <c r="D26" s="90"/>
-      <c r="E26" s="90"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="90"/>
-      <c r="H26" s="90"/>
-      <c r="I26" s="90"/>
-      <c r="J26" s="90"/>
-      <c r="K26" s="90"/>
-      <c r="L26" s="90"/>
-      <c r="M26" s="90"/>
-      <c r="N26" s="90"/>
-      <c r="O26" s="90"/>
-      <c r="P26" s="90"/>
-      <c r="Q26" s="90"/>
-      <c r="R26" s="90"/>
+      <c r="D26" s="98"/>
+      <c r="E26" s="98"/>
+      <c r="F26" s="98"/>
+      <c r="G26" s="98"/>
+      <c r="H26" s="98"/>
+      <c r="I26" s="98"/>
+      <c r="J26" s="98"/>
+      <c r="K26" s="98"/>
+      <c r="L26" s="98"/>
+      <c r="M26" s="98"/>
+      <c r="N26" s="98"/>
+      <c r="O26" s="98"/>
+      <c r="P26" s="98"/>
+      <c r="Q26" s="98"/>
+      <c r="R26" s="98"/>
       <c r="S26" s="65"/>
     </row>
     <row r="27" spans="2:19" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="45"/>
-      <c r="C27" s="91" t="s">
+      <c r="C27" s="117" t="s">
         <v>113</v>
       </c>
-      <c r="D27" s="91"/>
-      <c r="E27" s="91"/>
-      <c r="F27" s="91"/>
-      <c r="G27" s="91"/>
-      <c r="H27" s="91"/>
-      <c r="I27" s="91"/>
-      <c r="J27" s="91"/>
-      <c r="K27" s="91"/>
-      <c r="L27" s="91"/>
-      <c r="M27" s="91"/>
-      <c r="N27" s="91"/>
-      <c r="O27" s="91"/>
-      <c r="P27" s="91"/>
-      <c r="Q27" s="91"/>
-      <c r="R27" s="91"/>
+      <c r="D27" s="117"/>
+      <c r="E27" s="117"/>
+      <c r="F27" s="117"/>
+      <c r="G27" s="117"/>
+      <c r="H27" s="117"/>
+      <c r="I27" s="117"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="117"/>
+      <c r="L27" s="117"/>
+      <c r="M27" s="117"/>
+      <c r="N27" s="117"/>
+      <c r="O27" s="117"/>
+      <c r="P27" s="117"/>
+      <c r="Q27" s="117"/>
+      <c r="R27" s="117"/>
       <c r="S27" s="46"/>
     </row>
     <row r="28" spans="2:19" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="45"/>
-      <c r="C28" s="92"/>
-      <c r="D28" s="92"/>
-      <c r="E28" s="92"/>
-      <c r="F28" s="92"/>
-      <c r="G28" s="92"/>
-      <c r="H28" s="92"/>
-      <c r="I28" s="92"/>
-      <c r="J28" s="92"/>
-      <c r="K28" s="92"/>
-      <c r="L28" s="92"/>
-      <c r="M28" s="92"/>
-      <c r="N28" s="92"/>
-      <c r="O28" s="92"/>
-      <c r="P28" s="92"/>
-      <c r="Q28" s="92"/>
-      <c r="R28" s="92"/>
+      <c r="C28" s="118" t="s">
+        <v>150</v>
+      </c>
+      <c r="D28" s="118"/>
+      <c r="E28" s="118"/>
+      <c r="F28" s="118"/>
+      <c r="G28" s="118"/>
+      <c r="H28" s="118"/>
+      <c r="I28" s="118"/>
+      <c r="J28" s="118"/>
+      <c r="K28" s="118"/>
+      <c r="L28" s="118"/>
+      <c r="M28" s="118"/>
+      <c r="N28" s="118"/>
+      <c r="O28" s="118"/>
+      <c r="P28" s="118"/>
+      <c r="Q28" s="118"/>
+      <c r="R28" s="118"/>
       <c r="S28" s="46"/>
     </row>
     <row r="29" spans="2:19" ht="12" customHeight="1" x14ac:dyDescent="0.25">
@@ -4464,24 +4574,24 @@
     </row>
     <row r="30" spans="2:19" s="63" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="61"/>
-      <c r="C30" s="90" t="s">
+      <c r="C30" s="98" t="s">
         <v>122</v>
       </c>
-      <c r="D30" s="90"/>
-      <c r="E30" s="90"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="90"/>
-      <c r="H30" s="90"/>
-      <c r="I30" s="90"/>
-      <c r="J30" s="90"/>
-      <c r="K30" s="90"/>
-      <c r="L30" s="90"/>
-      <c r="M30" s="90"/>
-      <c r="N30" s="90"/>
-      <c r="O30" s="90"/>
-      <c r="P30" s="90"/>
-      <c r="Q30" s="90"/>
-      <c r="R30" s="90"/>
+      <c r="D30" s="98"/>
+      <c r="E30" s="98"/>
+      <c r="F30" s="98"/>
+      <c r="G30" s="98"/>
+      <c r="H30" s="98"/>
+      <c r="I30" s="98"/>
+      <c r="J30" s="98"/>
+      <c r="K30" s="98"/>
+      <c r="L30" s="98"/>
+      <c r="M30" s="98"/>
+      <c r="N30" s="98"/>
+      <c r="O30" s="98"/>
+      <c r="P30" s="98"/>
+      <c r="Q30" s="98"/>
+      <c r="R30" s="98"/>
       <c r="S30" s="65"/>
     </row>
     <row r="31" spans="2:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4520,30 +4630,30 @@
     </row>
     <row r="33" spans="2:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="45"/>
-      <c r="C33" s="94" t="s">
+      <c r="C33" s="110" t="s">
         <v>127</v>
       </c>
-      <c r="D33" s="95"/>
-      <c r="E33" s="80"/>
+      <c r="D33" s="111"/>
+      <c r="E33" s="76"/>
       <c r="F33" s="58"/>
-      <c r="G33" s="94" t="s">
+      <c r="G33" s="110" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="95"/>
-      <c r="I33" s="80"/>
+      <c r="H33" s="111"/>
+      <c r="I33" s="76"/>
       <c r="J33" s="58"/>
-      <c r="K33" s="94" t="s">
+      <c r="K33" s="110" t="s">
         <v>92</v>
       </c>
-      <c r="L33" s="95"/>
-      <c r="M33" s="104"/>
-      <c r="N33" s="105"/>
+      <c r="L33" s="111"/>
+      <c r="M33" s="86"/>
+      <c r="N33" s="87"/>
       <c r="O33" s="58"/>
-      <c r="P33" s="94" t="s">
+      <c r="P33" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="Q33" s="95"/>
-      <c r="R33" s="80" t="s">
+      <c r="Q33" s="111"/>
+      <c r="R33" s="76" t="s">
         <v>132</v>
       </c>
       <c r="S33" s="46"/>
@@ -4570,30 +4680,32 @@
     </row>
     <row r="35" spans="2:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="45"/>
-      <c r="C35" s="94" t="s">
+      <c r="C35" s="110" t="s">
         <v>136</v>
       </c>
-      <c r="D35" s="95"/>
-      <c r="E35" s="80"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="76"/>
       <c r="F35" s="58"/>
-      <c r="G35" s="94" t="s">
+      <c r="G35" s="110" t="s">
         <v>137</v>
       </c>
-      <c r="H35" s="95"/>
-      <c r="I35" s="80"/>
+      <c r="H35" s="111"/>
+      <c r="I35" s="76"/>
       <c r="J35" s="58"/>
-      <c r="K35" s="94" t="s">
+      <c r="K35" s="110" t="s">
         <v>93</v>
       </c>
-      <c r="L35" s="95"/>
-      <c r="M35" s="104"/>
-      <c r="N35" s="105"/>
+      <c r="L35" s="111"/>
+      <c r="M35" s="86"/>
+      <c r="N35" s="87"/>
       <c r="O35" s="58"/>
-      <c r="P35" s="94" t="s">
+      <c r="P35" s="110" t="s">
         <v>94</v>
       </c>
-      <c r="Q35" s="95"/>
-      <c r="R35" s="80"/>
+      <c r="Q35" s="111"/>
+      <c r="R35" s="76" t="s">
+        <v>131</v>
+      </c>
       <c r="S35" s="46"/>
     </row>
     <row r="36" spans="2:19" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4618,24 +4730,24 @@
     </row>
     <row r="37" spans="2:19" s="63" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="61"/>
-      <c r="C37" s="90" t="s">
+      <c r="C37" s="98" t="s">
         <v>105</v>
       </c>
-      <c r="D37" s="90"/>
-      <c r="E37" s="90"/>
-      <c r="F37" s="90"/>
-      <c r="G37" s="90"/>
-      <c r="H37" s="90"/>
-      <c r="I37" s="90"/>
-      <c r="J37" s="90"/>
-      <c r="K37" s="90"/>
-      <c r="L37" s="90"/>
-      <c r="M37" s="90"/>
-      <c r="N37" s="90"/>
-      <c r="O37" s="90"/>
-      <c r="P37" s="90"/>
-      <c r="Q37" s="90"/>
-      <c r="R37" s="90"/>
+      <c r="D37" s="98"/>
+      <c r="E37" s="98"/>
+      <c r="F37" s="98"/>
+      <c r="G37" s="98"/>
+      <c r="H37" s="98"/>
+      <c r="I37" s="98"/>
+      <c r="J37" s="98"/>
+      <c r="K37" s="98"/>
+      <c r="L37" s="98"/>
+      <c r="M37" s="98"/>
+      <c r="N37" s="98"/>
+      <c r="O37" s="98"/>
+      <c r="P37" s="98"/>
+      <c r="Q37" s="98"/>
+      <c r="R37" s="98"/>
       <c r="S37" s="65"/>
     </row>
     <row r="38" spans="2:19" ht="3" customHeight="1" x14ac:dyDescent="0.25">
@@ -4651,62 +4763,82 @@
     </row>
     <row r="40" spans="2:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="45"/>
-      <c r="C40" s="78" t="s">
+      <c r="C40" s="74" t="s">
         <v>129</v>
       </c>
-      <c r="D40" s="78" t="s">
+      <c r="D40" s="74" t="s">
         <v>116</v>
       </c>
-      <c r="E40" s="78" t="s">
+      <c r="E40" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="F40" s="93" t="s">
+      <c r="F40" s="107" t="s">
         <v>128</v>
       </c>
-      <c r="G40" s="93"/>
-      <c r="H40" s="93"/>
-      <c r="I40" s="93" t="s">
+      <c r="G40" s="107"/>
+      <c r="H40" s="107"/>
+      <c r="I40" s="107" t="s">
         <v>91</v>
       </c>
-      <c r="J40" s="93"/>
-      <c r="K40" s="101" t="s">
+      <c r="J40" s="107"/>
+      <c r="K40" s="112" t="s">
         <v>117</v>
       </c>
-      <c r="L40" s="102"/>
-      <c r="M40" s="93" t="s">
+      <c r="L40" s="113"/>
+      <c r="M40" s="107" t="s">
         <v>92</v>
       </c>
-      <c r="N40" s="93"/>
-      <c r="O40" s="78" t="s">
+      <c r="N40" s="107"/>
+      <c r="O40" s="74" t="s">
         <v>93</v>
       </c>
-      <c r="P40" s="78" t="s">
+      <c r="P40" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="Q40" s="93" t="s">
+      <c r="Q40" s="107" t="s">
         <v>98</v>
       </c>
-      <c r="R40" s="93"/>
+      <c r="R40" s="107"/>
       <c r="S40" s="46"/>
     </row>
-    <row r="41" spans="2:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="45"/>
-      <c r="C41" s="34"/>
-      <c r="D41" s="34"/>
-      <c r="E41" s="34"/>
-      <c r="F41" s="85"/>
-      <c r="G41" s="86"/>
-      <c r="H41" s="87"/>
-      <c r="I41" s="85"/>
-      <c r="J41" s="86"/>
-      <c r="K41" s="85"/>
-      <c r="L41" s="86"/>
-      <c r="M41" s="85"/>
-      <c r="N41" s="87"/>
-      <c r="O41" s="83"/>
-      <c r="P41" s="83"/>
-      <c r="Q41" s="85"/>
-      <c r="R41" s="87"/>
+      <c r="C41" s="34">
+        <v>8</v>
+      </c>
+      <c r="D41" s="34">
+        <v>10</v>
+      </c>
+      <c r="E41" s="34">
+        <v>7</v>
+      </c>
+      <c r="F41" s="149" t="s">
+        <v>151</v>
+      </c>
+      <c r="G41" s="150"/>
+      <c r="H41" s="151"/>
+      <c r="I41" s="149" t="s">
+        <v>152</v>
+      </c>
+      <c r="J41" s="150"/>
+      <c r="K41" s="149" t="s">
+        <v>149</v>
+      </c>
+      <c r="L41" s="150"/>
+      <c r="M41" s="149" t="s">
+        <v>153</v>
+      </c>
+      <c r="N41" s="151"/>
+      <c r="O41" s="79">
+        <v>1</v>
+      </c>
+      <c r="P41" s="79" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q41" s="149" t="s">
+        <v>155</v>
+      </c>
+      <c r="R41" s="151"/>
       <c r="S41" s="46"/>
     </row>
     <row r="42" spans="2:19" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4714,39 +4846,39 @@
       <c r="C42" s="34"/>
       <c r="D42" s="34"/>
       <c r="E42" s="34"/>
-      <c r="F42" s="85"/>
-      <c r="G42" s="86"/>
-      <c r="H42" s="87"/>
-      <c r="I42" s="85"/>
-      <c r="J42" s="87"/>
-      <c r="K42" s="85"/>
-      <c r="L42" s="87"/>
-      <c r="M42" s="85"/>
-      <c r="N42" s="87"/>
-      <c r="O42" s="83"/>
-      <c r="P42" s="83"/>
-      <c r="Q42" s="85"/>
-      <c r="R42" s="87"/>
+      <c r="F42" s="81"/>
+      <c r="G42" s="82"/>
+      <c r="H42" s="83"/>
+      <c r="I42" s="81"/>
+      <c r="J42" s="83"/>
+      <c r="K42" s="81"/>
+      <c r="L42" s="83"/>
+      <c r="M42" s="81"/>
+      <c r="N42" s="83"/>
+      <c r="O42" s="79"/>
+      <c r="P42" s="79"/>
+      <c r="Q42" s="81"/>
+      <c r="R42" s="83"/>
       <c r="S42" s="46"/>
     </row>
     <row r="43" spans="2:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="45"/>
       <c r="C43" s="34"/>
-      <c r="D43" s="82"/>
-      <c r="E43" s="82"/>
-      <c r="F43" s="85"/>
-      <c r="G43" s="86"/>
-      <c r="H43" s="87"/>
-      <c r="I43" s="85"/>
-      <c r="J43" s="86"/>
-      <c r="K43" s="85"/>
-      <c r="L43" s="87"/>
-      <c r="M43" s="85"/>
-      <c r="N43" s="99"/>
-      <c r="O43" s="83"/>
-      <c r="P43" s="83"/>
-      <c r="Q43" s="85"/>
-      <c r="R43" s="87"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="81"/>
+      <c r="G43" s="82"/>
+      <c r="H43" s="83"/>
+      <c r="I43" s="81"/>
+      <c r="J43" s="82"/>
+      <c r="K43" s="81"/>
+      <c r="L43" s="83"/>
+      <c r="M43" s="81"/>
+      <c r="N43" s="106"/>
+      <c r="O43" s="79"/>
+      <c r="P43" s="79"/>
+      <c r="Q43" s="81"/>
+      <c r="R43" s="83"/>
       <c r="S43" s="46"/>
     </row>
     <row r="44" spans="2:19" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4758,62 +4890,82 @@
     </row>
     <row r="45" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="45"/>
-      <c r="C45" s="78" t="s">
+      <c r="C45" s="74" t="s">
         <v>129</v>
       </c>
-      <c r="D45" s="78" t="s">
+      <c r="D45" s="74" t="s">
         <v>116</v>
       </c>
-      <c r="E45" s="78" t="s">
+      <c r="E45" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="F45" s="93" t="s">
+      <c r="F45" s="107" t="s">
         <v>128</v>
       </c>
-      <c r="G45" s="93"/>
-      <c r="H45" s="93"/>
-      <c r="I45" s="93" t="s">
+      <c r="G45" s="107"/>
+      <c r="H45" s="107"/>
+      <c r="I45" s="107" t="s">
         <v>91</v>
       </c>
-      <c r="J45" s="93"/>
-      <c r="K45" s="101" t="s">
+      <c r="J45" s="107"/>
+      <c r="K45" s="112" t="s">
         <v>117</v>
       </c>
-      <c r="L45" s="102"/>
-      <c r="M45" s="93" t="s">
+      <c r="L45" s="113"/>
+      <c r="M45" s="107" t="s">
         <v>92</v>
       </c>
-      <c r="N45" s="93"/>
-      <c r="O45" s="78" t="s">
+      <c r="N45" s="107"/>
+      <c r="O45" s="74" t="s">
         <v>93</v>
       </c>
-      <c r="P45" s="78" t="s">
+      <c r="P45" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="Q45" s="93" t="s">
+      <c r="Q45" s="107" t="s">
         <v>98</v>
       </c>
-      <c r="R45" s="93"/>
+      <c r="R45" s="107"/>
       <c r="S45" s="46"/>
     </row>
-    <row r="46" spans="2:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:19" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="45"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="34"/>
-      <c r="E46" s="34"/>
-      <c r="F46" s="85"/>
-      <c r="G46" s="86"/>
-      <c r="H46" s="87"/>
-      <c r="I46" s="85"/>
-      <c r="J46" s="86"/>
-      <c r="K46" s="85"/>
-      <c r="L46" s="86"/>
-      <c r="M46" s="85"/>
-      <c r="N46" s="87"/>
-      <c r="O46" s="83"/>
-      <c r="P46" s="83"/>
-      <c r="Q46" s="85"/>
-      <c r="R46" s="87"/>
+      <c r="C46" s="34">
+        <v>8</v>
+      </c>
+      <c r="D46" s="34">
+        <v>10</v>
+      </c>
+      <c r="E46" s="34">
+        <v>7</v>
+      </c>
+      <c r="F46" s="149" t="s">
+        <v>151</v>
+      </c>
+      <c r="G46" s="150"/>
+      <c r="H46" s="151"/>
+      <c r="I46" s="149" t="s">
+        <v>152</v>
+      </c>
+      <c r="J46" s="150"/>
+      <c r="K46" s="149" t="s">
+        <v>149</v>
+      </c>
+      <c r="L46" s="150"/>
+      <c r="M46" s="149" t="s">
+        <v>153</v>
+      </c>
+      <c r="N46" s="151"/>
+      <c r="O46" s="79">
+        <v>1</v>
+      </c>
+      <c r="P46" s="79" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q46" s="149" t="s">
+        <v>164</v>
+      </c>
+      <c r="R46" s="151"/>
       <c r="S46" s="46"/>
     </row>
     <row r="47" spans="2:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4821,101 +4973,101 @@
       <c r="C47" s="34"/>
       <c r="D47" s="34"/>
       <c r="E47" s="34"/>
-      <c r="F47" s="85"/>
-      <c r="G47" s="86"/>
-      <c r="H47" s="87"/>
-      <c r="I47" s="88"/>
-      <c r="J47" s="89"/>
-      <c r="K47" s="85"/>
-      <c r="L47" s="87"/>
-      <c r="M47" s="85"/>
-      <c r="N47" s="87"/>
-      <c r="O47" s="83"/>
-      <c r="P47" s="83"/>
-      <c r="Q47" s="85"/>
-      <c r="R47" s="87"/>
+      <c r="F47" s="81"/>
+      <c r="G47" s="82"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="119"/>
+      <c r="J47" s="120"/>
+      <c r="K47" s="81"/>
+      <c r="L47" s="83"/>
+      <c r="M47" s="81"/>
+      <c r="N47" s="83"/>
+      <c r="O47" s="79"/>
+      <c r="P47" s="79"/>
+      <c r="Q47" s="81"/>
+      <c r="R47" s="83"/>
       <c r="S47" s="46"/>
     </row>
     <row r="48" spans="2:19" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="45"/>
-      <c r="C48" s="82"/>
-      <c r="D48" s="82"/>
-      <c r="E48" s="82"/>
-      <c r="F48" s="85"/>
-      <c r="G48" s="86"/>
-      <c r="H48" s="87"/>
-      <c r="I48" s="85"/>
-      <c r="J48" s="86"/>
-      <c r="K48" s="85"/>
-      <c r="L48" s="87"/>
-      <c r="M48" s="85"/>
-      <c r="N48" s="99"/>
-      <c r="O48" s="83"/>
-      <c r="P48" s="83"/>
-      <c r="Q48" s="85"/>
-      <c r="R48" s="87"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="81"/>
+      <c r="G48" s="82"/>
+      <c r="H48" s="83"/>
+      <c r="I48" s="81"/>
+      <c r="J48" s="82"/>
+      <c r="K48" s="81"/>
+      <c r="L48" s="83"/>
+      <c r="M48" s="81"/>
+      <c r="N48" s="106"/>
+      <c r="O48" s="79"/>
+      <c r="P48" s="79"/>
+      <c r="Q48" s="81"/>
+      <c r="R48" s="83"/>
       <c r="S48" s="46"/>
     </row>
     <row r="49" spans="2:19" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="45"/>
-      <c r="C49" s="112"/>
-      <c r="D49" s="112"/>
-      <c r="E49" s="112"/>
-      <c r="F49" s="112"/>
-      <c r="G49" s="112"/>
-      <c r="H49" s="112"/>
-      <c r="I49" s="112"/>
-      <c r="J49" s="112"/>
-      <c r="K49" s="112"/>
-      <c r="L49" s="112"/>
-      <c r="M49" s="112"/>
-      <c r="N49" s="112"/>
-      <c r="O49" s="112"/>
-      <c r="P49" s="112"/>
-      <c r="Q49" s="112"/>
-      <c r="R49" s="112"/>
+      <c r="C49" s="105"/>
+      <c r="D49" s="105"/>
+      <c r="E49" s="105"/>
+      <c r="F49" s="105"/>
+      <c r="G49" s="105"/>
+      <c r="H49" s="105"/>
+      <c r="I49" s="105"/>
+      <c r="J49" s="105"/>
+      <c r="K49" s="105"/>
+      <c r="L49" s="105"/>
+      <c r="M49" s="105"/>
+      <c r="N49" s="105"/>
+      <c r="O49" s="105"/>
+      <c r="P49" s="105"/>
+      <c r="Q49" s="105"/>
+      <c r="R49" s="105"/>
       <c r="S49" s="46"/>
     </row>
     <row r="50" spans="2:19" s="63" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="61"/>
-      <c r="C50" s="90" t="s">
+      <c r="C50" s="98" t="s">
         <v>106</v>
       </c>
-      <c r="D50" s="90"/>
-      <c r="E50" s="90"/>
-      <c r="F50" s="90"/>
-      <c r="G50" s="90"/>
-      <c r="H50" s="90"/>
-      <c r="I50" s="90"/>
-      <c r="J50" s="90"/>
-      <c r="K50" s="90"/>
-      <c r="L50" s="90"/>
-      <c r="M50" s="90"/>
-      <c r="N50" s="90"/>
-      <c r="O50" s="90"/>
-      <c r="P50" s="90"/>
-      <c r="Q50" s="90"/>
-      <c r="R50" s="90"/>
+      <c r="D50" s="98"/>
+      <c r="E50" s="98"/>
+      <c r="F50" s="98"/>
+      <c r="G50" s="98"/>
+      <c r="H50" s="98"/>
+      <c r="I50" s="98"/>
+      <c r="J50" s="98"/>
+      <c r="K50" s="98"/>
+      <c r="L50" s="98"/>
+      <c r="M50" s="98"/>
+      <c r="N50" s="98"/>
+      <c r="O50" s="98"/>
+      <c r="P50" s="98"/>
+      <c r="Q50" s="98"/>
+      <c r="R50" s="98"/>
       <c r="S50" s="65"/>
     </row>
     <row r="51" spans="2:19" ht="3" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="45"/>
-      <c r="C51" s="97"/>
-      <c r="D51" s="97"/>
-      <c r="E51" s="97"/>
-      <c r="F51" s="97"/>
-      <c r="G51" s="97"/>
-      <c r="H51" s="97"/>
-      <c r="I51" s="97"/>
-      <c r="J51" s="97"/>
-      <c r="K51" s="97"/>
-      <c r="L51" s="97"/>
-      <c r="M51" s="97"/>
-      <c r="N51" s="97"/>
-      <c r="O51" s="97"/>
-      <c r="P51" s="97"/>
-      <c r="Q51" s="97"/>
-      <c r="R51" s="97"/>
+      <c r="C51" s="115"/>
+      <c r="D51" s="115"/>
+      <c r="E51" s="115"/>
+      <c r="F51" s="115"/>
+      <c r="G51" s="115"/>
+      <c r="H51" s="115"/>
+      <c r="I51" s="115"/>
+      <c r="J51" s="115"/>
+      <c r="K51" s="115"/>
+      <c r="L51" s="115"/>
+      <c r="M51" s="115"/>
+      <c r="N51" s="115"/>
+      <c r="O51" s="115"/>
+      <c r="P51" s="115"/>
+      <c r="Q51" s="115"/>
+      <c r="R51" s="115"/>
       <c r="S51" s="46"/>
     </row>
     <row r="52" spans="2:19" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4927,42 +5079,42 @@
     </row>
     <row r="53" spans="2:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="45"/>
-      <c r="C53" s="96"/>
-      <c r="D53" s="96"/>
-      <c r="E53" s="96"/>
-      <c r="F53" s="96"/>
-      <c r="G53" s="96"/>
-      <c r="H53" s="96"/>
-      <c r="I53" s="96"/>
-      <c r="J53" s="96"/>
-      <c r="K53" s="96"/>
-      <c r="L53" s="96"/>
-      <c r="M53" s="96"/>
-      <c r="N53" s="96"/>
-      <c r="O53" s="96"/>
-      <c r="P53" s="96"/>
-      <c r="Q53" s="96"/>
-      <c r="R53" s="96"/>
+      <c r="C53" s="114"/>
+      <c r="D53" s="114"/>
+      <c r="E53" s="114"/>
+      <c r="F53" s="114"/>
+      <c r="G53" s="114"/>
+      <c r="H53" s="114"/>
+      <c r="I53" s="114"/>
+      <c r="J53" s="114"/>
+      <c r="K53" s="114"/>
+      <c r="L53" s="114"/>
+      <c r="M53" s="114"/>
+      <c r="N53" s="114"/>
+      <c r="O53" s="114"/>
+      <c r="P53" s="114"/>
+      <c r="Q53" s="114"/>
+      <c r="R53" s="114"/>
       <c r="S53" s="46"/>
     </row>
     <row r="54" spans="2:19" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="45"/>
-      <c r="C54" s="106"/>
-      <c r="D54" s="107"/>
-      <c r="E54" s="107"/>
-      <c r="F54" s="107"/>
-      <c r="G54" s="108"/>
-      <c r="H54" s="106"/>
-      <c r="I54" s="107"/>
-      <c r="J54" s="107"/>
-      <c r="K54" s="107"/>
-      <c r="L54" s="108"/>
-      <c r="M54" s="113"/>
-      <c r="N54" s="113"/>
-      <c r="O54" s="113"/>
-      <c r="P54" s="113"/>
-      <c r="Q54" s="113"/>
-      <c r="R54" s="113"/>
+      <c r="C54" s="99"/>
+      <c r="D54" s="100"/>
+      <c r="E54" s="100"/>
+      <c r="F54" s="100"/>
+      <c r="G54" s="101"/>
+      <c r="H54" s="99"/>
+      <c r="I54" s="100"/>
+      <c r="J54" s="100"/>
+      <c r="K54" s="100"/>
+      <c r="L54" s="101"/>
+      <c r="M54" s="108"/>
+      <c r="N54" s="108"/>
+      <c r="O54" s="108"/>
+      <c r="P54" s="108"/>
+      <c r="Q54" s="108"/>
+      <c r="R54" s="108"/>
       <c r="S54" s="46"/>
     </row>
     <row r="55" spans="2:19" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4987,6 +5139,72 @@
     </row>
   </sheetData>
   <mergeCells count="82">
+    <mergeCell ref="F47:H47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="Q47:R47"/>
+    <mergeCell ref="F42:H42"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="M42:N42"/>
+    <mergeCell ref="Q42:R42"/>
+    <mergeCell ref="C26:R26"/>
+    <mergeCell ref="C27:R27"/>
+    <mergeCell ref="C28:R28"/>
+    <mergeCell ref="C30:R30"/>
+    <mergeCell ref="Q40:R40"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="M40:N40"/>
+    <mergeCell ref="P33:Q33"/>
+    <mergeCell ref="C50:R50"/>
+    <mergeCell ref="C53:R53"/>
+    <mergeCell ref="C51:R51"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="M41:N41"/>
+    <mergeCell ref="Q41:R41"/>
+    <mergeCell ref="Q46:R46"/>
+    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="Q45:R45"/>
+    <mergeCell ref="Q43:R43"/>
+    <mergeCell ref="M43:N43"/>
+    <mergeCell ref="F45:H45"/>
+    <mergeCell ref="C37:R37"/>
+    <mergeCell ref="C3:R3"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="H54:L54"/>
+    <mergeCell ref="C54:G54"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="K46:L46"/>
+    <mergeCell ref="C49:R49"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="M48:N48"/>
+    <mergeCell ref="Q48:R48"/>
+    <mergeCell ref="K48:L48"/>
+    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="M54:R54"/>
     <mergeCell ref="I46:J46"/>
     <mergeCell ref="M46:N46"/>
     <mergeCell ref="C5:R5"/>
@@ -5003,72 +5221,6 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:G8"/>
     <mergeCell ref="C22:R22"/>
-    <mergeCell ref="H54:L54"/>
-    <mergeCell ref="C54:G54"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="K46:L46"/>
-    <mergeCell ref="C49:R49"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="M48:N48"/>
-    <mergeCell ref="Q48:R48"/>
-    <mergeCell ref="K48:L48"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="M54:R54"/>
-    <mergeCell ref="C3:R3"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="K45:L45"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="F40:H40"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="C50:R50"/>
-    <mergeCell ref="C53:R53"/>
-    <mergeCell ref="C51:R51"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="F41:H41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="M41:N41"/>
-    <mergeCell ref="Q41:R41"/>
-    <mergeCell ref="Q46:R46"/>
-    <mergeCell ref="F43:H43"/>
-    <mergeCell ref="Q45:R45"/>
-    <mergeCell ref="Q43:R43"/>
-    <mergeCell ref="M43:N43"/>
-    <mergeCell ref="F45:H45"/>
-    <mergeCell ref="C37:R37"/>
-    <mergeCell ref="C26:R26"/>
-    <mergeCell ref="C27:R27"/>
-    <mergeCell ref="C28:R28"/>
-    <mergeCell ref="C30:R30"/>
-    <mergeCell ref="Q40:R40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="M40:N40"/>
-    <mergeCell ref="P33:Q33"/>
-    <mergeCell ref="F42:H42"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="K42:L42"/>
-    <mergeCell ref="M42:N42"/>
-    <mergeCell ref="Q42:R42"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="Q47:R47"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G31:H31 G25:H25 G29:H29" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -5137,63 +5289,63 @@
     </row>
     <row r="3" spans="2:18" ht="3.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="45"/>
-      <c r="C3" s="100"/>
-      <c r="D3" s="100"/>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="100"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="100"/>
-      <c r="L3" s="100"/>
-      <c r="M3" s="100"/>
-      <c r="N3" s="100"/>
-      <c r="O3" s="100"/>
-      <c r="P3" s="100"/>
-      <c r="Q3" s="100"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="109"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="109"/>
+      <c r="H3" s="109"/>
+      <c r="I3" s="109"/>
+      <c r="J3" s="109"/>
+      <c r="K3" s="109"/>
+      <c r="L3" s="109"/>
+      <c r="M3" s="109"/>
+      <c r="N3" s="109"/>
+      <c r="O3" s="109"/>
+      <c r="P3" s="109"/>
+      <c r="Q3" s="109"/>
       <c r="R3" s="46"/>
     </row>
     <row r="4" spans="2:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="45"/>
-      <c r="C4" s="115" t="s">
+      <c r="C4" s="85" t="s">
         <v>133</v>
       </c>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="85"/>
+      <c r="I4" s="85"/>
+      <c r="J4" s="85"/>
+      <c r="K4" s="85"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="85"/>
+      <c r="O4" s="85"/>
+      <c r="P4" s="85"/>
+      <c r="Q4" s="85"/>
       <c r="R4" s="46"/>
     </row>
     <row r="5" spans="2:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="45"/>
-      <c r="C5" s="150" t="s">
+      <c r="C5" s="136" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="150"/>
-      <c r="E5" s="150"/>
-      <c r="F5" s="150"/>
-      <c r="G5" s="150"/>
-      <c r="H5" s="150"/>
-      <c r="I5" s="150"/>
-      <c r="J5" s="150"/>
-      <c r="K5" s="150"/>
-      <c r="L5" s="150"/>
-      <c r="M5" s="150"/>
-      <c r="N5" s="150"/>
-      <c r="O5" s="150"/>
-      <c r="P5" s="150"/>
-      <c r="Q5" s="150"/>
+      <c r="D5" s="136"/>
+      <c r="E5" s="136"/>
+      <c r="F5" s="136"/>
+      <c r="G5" s="136"/>
+      <c r="H5" s="136"/>
+      <c r="I5" s="136"/>
+      <c r="J5" s="136"/>
+      <c r="K5" s="136"/>
+      <c r="L5" s="136"/>
+      <c r="M5" s="136"/>
+      <c r="N5" s="136"/>
+      <c r="O5" s="136"/>
+      <c r="P5" s="136"/>
+      <c r="Q5" s="136"/>
       <c r="R5" s="46"/>
     </row>
     <row r="6" spans="2:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5215,11 +5367,11 @@
       <c r="N7" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="O7" s="153" t="s">
-        <v>143</v>
-      </c>
-      <c r="P7" s="154"/>
-      <c r="Q7" s="155"/>
+      <c r="O7" s="139" t="s">
+        <v>158</v>
+      </c>
+      <c r="P7" s="140"/>
+      <c r="Q7" s="141"/>
       <c r="R7" s="46"/>
     </row>
     <row r="8" spans="2:18" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5243,16 +5395,16 @@
     </row>
     <row r="9" spans="2:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="45"/>
-      <c r="C9" s="121" t="s">
+      <c r="C9" s="94" t="s">
         <v>114</v>
       </c>
-      <c r="D9" s="121"/>
-      <c r="E9" s="121"/>
-      <c r="F9" s="151">
-        <v>46275</v>
-      </c>
-      <c r="G9" s="152"/>
-      <c r="H9" s="152"/>
+      <c r="D9" s="94"/>
+      <c r="E9" s="94"/>
+      <c r="F9" s="137">
+        <v>46091</v>
+      </c>
+      <c r="G9" s="138"/>
+      <c r="H9" s="138"/>
       <c r="I9" s="26"/>
       <c r="J9" s="26"/>
       <c r="K9" s="26"/>
@@ -5277,23 +5429,23 @@
     </row>
     <row r="11" spans="2:18" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="45"/>
-      <c r="C11" s="149" t="s">
+      <c r="C11" s="135" t="s">
         <v>138</v>
       </c>
-      <c r="D11" s="149"/>
-      <c r="E11" s="149"/>
-      <c r="F11" s="149"/>
-      <c r="G11" s="149"/>
-      <c r="H11" s="149"/>
-      <c r="I11" s="149"/>
-      <c r="J11" s="149"/>
-      <c r="K11" s="149"/>
-      <c r="L11" s="149"/>
-      <c r="M11" s="149"/>
-      <c r="N11" s="149"/>
-      <c r="O11" s="149"/>
-      <c r="P11" s="149"/>
-      <c r="Q11" s="149"/>
+      <c r="D11" s="135"/>
+      <c r="E11" s="135"/>
+      <c r="F11" s="135"/>
+      <c r="G11" s="135"/>
+      <c r="H11" s="135"/>
+      <c r="I11" s="135"/>
+      <c r="J11" s="135"/>
+      <c r="K11" s="135"/>
+      <c r="L11" s="135"/>
+      <c r="M11" s="135"/>
+      <c r="N11" s="135"/>
+      <c r="O11" s="135"/>
+      <c r="P11" s="135"/>
+      <c r="Q11" s="135"/>
       <c r="R11" s="46"/>
     </row>
     <row r="12" spans="2:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5326,25 +5478,25 @@
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="45"/>
-      <c r="C15" s="129" t="s">
+      <c r="C15" s="134" t="s">
         <v>107</v>
       </c>
-      <c r="D15" s="129"/>
-      <c r="E15" s="129"/>
-      <c r="F15" s="129"/>
+      <c r="D15" s="134"/>
+      <c r="E15" s="134"/>
+      <c r="F15" s="134"/>
       <c r="G15" s="20"/>
-      <c r="H15" s="130" t="s">
-        <v>144</v>
-      </c>
-      <c r="I15" s="131"/>
-      <c r="J15" s="131"/>
-      <c r="K15" s="131"/>
-      <c r="L15" s="131"/>
-      <c r="M15" s="131"/>
-      <c r="N15" s="131"/>
-      <c r="O15" s="131"/>
-      <c r="P15" s="131"/>
-      <c r="Q15" s="132"/>
+      <c r="H15" s="142" t="s">
+        <v>143</v>
+      </c>
+      <c r="I15" s="143"/>
+      <c r="J15" s="143"/>
+      <c r="K15" s="143"/>
+      <c r="L15" s="143"/>
+      <c r="M15" s="143"/>
+      <c r="N15" s="143"/>
+      <c r="O15" s="143"/>
+      <c r="P15" s="143"/>
+      <c r="Q15" s="144"/>
       <c r="R15" s="46"/>
     </row>
     <row r="16" spans="2:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5368,25 +5520,25 @@
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B17" s="45"/>
-      <c r="C17" s="129" t="s">
+      <c r="C17" s="134" t="s">
         <v>3</v>
       </c>
-      <c r="D17" s="129"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="129"/>
+      <c r="D17" s="134"/>
+      <c r="E17" s="134"/>
+      <c r="F17" s="134"/>
       <c r="G17" s="20"/>
-      <c r="H17" s="130" t="s">
-        <v>145</v>
-      </c>
-      <c r="I17" s="131"/>
-      <c r="J17" s="131"/>
-      <c r="K17" s="131"/>
-      <c r="L17" s="131"/>
-      <c r="M17" s="131"/>
-      <c r="N17" s="131"/>
-      <c r="O17" s="131"/>
-      <c r="P17" s="131"/>
-      <c r="Q17" s="132"/>
+      <c r="H17" s="142" t="s">
+        <v>144</v>
+      </c>
+      <c r="I17" s="143"/>
+      <c r="J17" s="143"/>
+      <c r="K17" s="143"/>
+      <c r="L17" s="143"/>
+      <c r="M17" s="143"/>
+      <c r="N17" s="143"/>
+      <c r="O17" s="143"/>
+      <c r="P17" s="143"/>
+      <c r="Q17" s="144"/>
       <c r="R17" s="46"/>
     </row>
     <row r="18" spans="2:18" ht="3" customHeight="1" x14ac:dyDescent="0.25">
@@ -5410,25 +5562,25 @@
     </row>
     <row r="19" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B19" s="45"/>
-      <c r="C19" s="129" t="s">
+      <c r="C19" s="134" t="s">
         <v>139</v>
       </c>
-      <c r="D19" s="129"/>
-      <c r="E19" s="129"/>
-      <c r="F19" s="129"/>
+      <c r="D19" s="134"/>
+      <c r="E19" s="134"/>
+      <c r="F19" s="134"/>
       <c r="G19" s="38"/>
-      <c r="H19" s="130" t="s">
-        <v>146</v>
-      </c>
-      <c r="I19" s="131"/>
-      <c r="J19" s="131"/>
-      <c r="K19" s="131"/>
-      <c r="L19" s="131"/>
-      <c r="M19" s="131"/>
-      <c r="N19" s="131"/>
-      <c r="O19" s="131"/>
-      <c r="P19" s="131"/>
-      <c r="Q19" s="132"/>
+      <c r="H19" s="142" t="s">
+        <v>145</v>
+      </c>
+      <c r="I19" s="143"/>
+      <c r="J19" s="143"/>
+      <c r="K19" s="143"/>
+      <c r="L19" s="143"/>
+      <c r="M19" s="143"/>
+      <c r="N19" s="143"/>
+      <c r="O19" s="143"/>
+      <c r="P19" s="143"/>
+      <c r="Q19" s="144"/>
       <c r="R19" s="46"/>
     </row>
     <row r="20" spans="2:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5452,25 +5604,25 @@
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B21" s="45"/>
-      <c r="C21" s="129" t="s">
+      <c r="C21" s="134" t="s">
         <v>125</v>
       </c>
-      <c r="D21" s="129"/>
-      <c r="E21" s="129"/>
-      <c r="F21" s="129"/>
+      <c r="D21" s="134"/>
+      <c r="E21" s="134"/>
+      <c r="F21" s="134"/>
       <c r="G21" s="38"/>
-      <c r="H21" s="130" t="s">
-        <v>147</v>
-      </c>
-      <c r="I21" s="131"/>
-      <c r="J21" s="131"/>
-      <c r="K21" s="131"/>
-      <c r="L21" s="131"/>
-      <c r="M21" s="131"/>
-      <c r="N21" s="131"/>
-      <c r="O21" s="131"/>
-      <c r="P21" s="131"/>
-      <c r="Q21" s="132"/>
+      <c r="H21" s="142" t="s">
+        <v>149</v>
+      </c>
+      <c r="I21" s="143"/>
+      <c r="J21" s="143"/>
+      <c r="K21" s="143"/>
+      <c r="L21" s="143"/>
+      <c r="M21" s="143"/>
+      <c r="N21" s="143"/>
+      <c r="O21" s="143"/>
+      <c r="P21" s="143"/>
+      <c r="Q21" s="144"/>
       <c r="R21" s="46"/>
     </row>
     <row r="22" spans="2:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5491,23 +5643,23 @@
     </row>
     <row r="23" spans="2:18" s="63" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="61"/>
-      <c r="C23" s="90" t="s">
+      <c r="C23" s="98" t="s">
         <v>112</v>
       </c>
-      <c r="D23" s="90"/>
-      <c r="E23" s="90"/>
-      <c r="F23" s="90"/>
-      <c r="G23" s="90"/>
-      <c r="H23" s="90"/>
-      <c r="I23" s="90"/>
-      <c r="J23" s="90"/>
-      <c r="K23" s="90"/>
-      <c r="L23" s="90"/>
-      <c r="M23" s="90"/>
-      <c r="N23" s="90"/>
-      <c r="O23" s="90"/>
-      <c r="P23" s="90"/>
-      <c r="Q23" s="90"/>
+      <c r="D23" s="98"/>
+      <c r="E23" s="98"/>
+      <c r="F23" s="98"/>
+      <c r="G23" s="98"/>
+      <c r="H23" s="98"/>
+      <c r="I23" s="98"/>
+      <c r="J23" s="98"/>
+      <c r="K23" s="98"/>
+      <c r="L23" s="98"/>
+      <c r="M23" s="98"/>
+      <c r="N23" s="98"/>
+      <c r="O23" s="98"/>
+      <c r="P23" s="98"/>
+      <c r="Q23" s="98"/>
       <c r="R23" s="65"/>
     </row>
     <row r="24" spans="2:18" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5531,28 +5683,30 @@
     </row>
     <row r="25" spans="2:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B25" s="45"/>
-      <c r="D25" s="134" t="s">
+      <c r="D25" s="130" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="135"/>
-      <c r="F25" s="98"/>
-      <c r="G25" s="98"/>
-      <c r="H25" s="146" t="s">
+      <c r="E25" s="131"/>
+      <c r="F25" s="116" t="s">
+        <v>131</v>
+      </c>
+      <c r="G25" s="116"/>
+      <c r="H25" s="129" t="s">
         <v>120</v>
       </c>
-      <c r="I25" s="134"/>
-      <c r="J25" s="134"/>
-      <c r="K25" s="135"/>
-      <c r="L25" s="147"/>
-      <c r="M25" s="147"/>
-      <c r="N25" s="134" t="s">
+      <c r="I25" s="130"/>
+      <c r="J25" s="130"/>
+      <c r="K25" s="131"/>
+      <c r="L25" s="132"/>
+      <c r="M25" s="132"/>
+      <c r="N25" s="130" t="s">
         <v>109</v>
       </c>
-      <c r="O25" s="135"/>
-      <c r="P25" s="148" t="s">
+      <c r="O25" s="131"/>
+      <c r="P25" s="133" t="s">
         <v>131</v>
       </c>
-      <c r="Q25" s="148"/>
+      <c r="Q25" s="133"/>
       <c r="R25" s="46"/>
     </row>
     <row r="26" spans="2:18" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5568,65 +5722,65 @@
     </row>
     <row r="27" spans="2:18" s="63" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="61"/>
-      <c r="C27" s="90" t="s">
+      <c r="C27" s="98" t="s">
         <v>104</v>
       </c>
-      <c r="D27" s="90"/>
-      <c r="E27" s="90"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="90"/>
-      <c r="H27" s="90"/>
-      <c r="I27" s="90"/>
-      <c r="J27" s="90"/>
-      <c r="K27" s="90"/>
-      <c r="L27" s="90"/>
-      <c r="M27" s="90"/>
-      <c r="N27" s="90"/>
-      <c r="O27" s="90"/>
-      <c r="P27" s="90"/>
-      <c r="Q27" s="90"/>
+      <c r="D27" s="98"/>
+      <c r="E27" s="98"/>
+      <c r="F27" s="98"/>
+      <c r="G27" s="98"/>
+      <c r="H27" s="98"/>
+      <c r="I27" s="98"/>
+      <c r="J27" s="98"/>
+      <c r="K27" s="98"/>
+      <c r="L27" s="98"/>
+      <c r="M27" s="98"/>
+      <c r="N27" s="98"/>
+      <c r="O27" s="98"/>
+      <c r="P27" s="98"/>
+      <c r="Q27" s="98"/>
       <c r="R27" s="65"/>
     </row>
     <row r="28" spans="2:18" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="45"/>
-      <c r="C28" s="91" t="s">
+      <c r="C28" s="117" t="s">
         <v>113</v>
       </c>
-      <c r="D28" s="91"/>
-      <c r="E28" s="91"/>
-      <c r="F28" s="91"/>
-      <c r="G28" s="91"/>
-      <c r="H28" s="91"/>
-      <c r="I28" s="91"/>
-      <c r="J28" s="91"/>
-      <c r="K28" s="91"/>
-      <c r="L28" s="91"/>
-      <c r="M28" s="91"/>
-      <c r="N28" s="91"/>
-      <c r="O28" s="91"/>
-      <c r="P28" s="91"/>
-      <c r="Q28" s="91"/>
+      <c r="D28" s="117"/>
+      <c r="E28" s="117"/>
+      <c r="F28" s="117"/>
+      <c r="G28" s="117"/>
+      <c r="H28" s="117"/>
+      <c r="I28" s="117"/>
+      <c r="J28" s="117"/>
+      <c r="K28" s="117"/>
+      <c r="L28" s="117"/>
+      <c r="M28" s="117"/>
+      <c r="N28" s="117"/>
+      <c r="O28" s="117"/>
+      <c r="P28" s="117"/>
+      <c r="Q28" s="117"/>
       <c r="R28" s="46"/>
     </row>
     <row r="29" spans="2:18" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="45"/>
-      <c r="C29" s="133" t="s">
-        <v>148</v>
-      </c>
-      <c r="D29" s="133"/>
-      <c r="E29" s="133"/>
-      <c r="F29" s="133"/>
-      <c r="G29" s="133"/>
-      <c r="H29" s="133"/>
-      <c r="I29" s="133"/>
-      <c r="J29" s="133"/>
-      <c r="K29" s="133"/>
-      <c r="L29" s="133"/>
-      <c r="M29" s="133"/>
-      <c r="N29" s="133"/>
-      <c r="O29" s="133"/>
-      <c r="P29" s="133"/>
-      <c r="Q29" s="133"/>
+      <c r="C29" s="148" t="s">
+        <v>159</v>
+      </c>
+      <c r="D29" s="148"/>
+      <c r="E29" s="148"/>
+      <c r="F29" s="148"/>
+      <c r="G29" s="148"/>
+      <c r="H29" s="148"/>
+      <c r="I29" s="148"/>
+      <c r="J29" s="148"/>
+      <c r="K29" s="148"/>
+      <c r="L29" s="148"/>
+      <c r="M29" s="148"/>
+      <c r="N29" s="148"/>
+      <c r="O29" s="148"/>
+      <c r="P29" s="148"/>
+      <c r="Q29" s="148"/>
       <c r="R29" s="46"/>
     </row>
     <row r="30" spans="2:18" ht="6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5639,23 +5793,23 @@
     </row>
     <row r="31" spans="2:18" s="63" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="61"/>
-      <c r="C31" s="90" t="s">
+      <c r="C31" s="98" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="90"/>
-      <c r="E31" s="90"/>
-      <c r="F31" s="90"/>
-      <c r="G31" s="90"/>
-      <c r="H31" s="90"/>
-      <c r="I31" s="90"/>
-      <c r="J31" s="90"/>
-      <c r="K31" s="90"/>
-      <c r="L31" s="90"/>
-      <c r="M31" s="90"/>
-      <c r="N31" s="90"/>
-      <c r="O31" s="90"/>
-      <c r="P31" s="90"/>
-      <c r="Q31" s="90"/>
+      <c r="D31" s="98"/>
+      <c r="E31" s="98"/>
+      <c r="F31" s="98"/>
+      <c r="G31" s="98"/>
+      <c r="H31" s="98"/>
+      <c r="I31" s="98"/>
+      <c r="J31" s="98"/>
+      <c r="K31" s="98"/>
+      <c r="L31" s="98"/>
+      <c r="M31" s="98"/>
+      <c r="N31" s="98"/>
+      <c r="O31" s="98"/>
+      <c r="P31" s="98"/>
+      <c r="Q31" s="98"/>
       <c r="R31" s="65"/>
     </row>
     <row r="32" spans="2:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5671,34 +5825,34 @@
     </row>
     <row r="33" spans="2:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="45"/>
-      <c r="C33" s="94" t="s">
+      <c r="C33" s="110" t="s">
         <v>130</v>
       </c>
-      <c r="D33" s="156"/>
-      <c r="E33" s="95"/>
+      <c r="D33" s="126"/>
+      <c r="E33" s="111"/>
       <c r="F33" s="34" t="s">
         <v>131</v>
       </c>
       <c r="G33" s="32"/>
-      <c r="H33" s="94" t="s">
+      <c r="H33" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="I33" s="95"/>
+      <c r="I33" s="111"/>
       <c r="J33" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="K33" s="94" t="s">
+      <c r="K33" s="110" t="s">
         <v>1</v>
       </c>
-      <c r="L33" s="95"/>
+      <c r="L33" s="111"/>
       <c r="M33" s="34" t="s">
         <v>131</v>
       </c>
       <c r="N33" s="32"/>
-      <c r="O33" s="94" t="s">
+      <c r="O33" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="P33" s="95"/>
+      <c r="P33" s="111"/>
       <c r="Q33" s="34" t="s">
         <v>131</v>
       </c>
@@ -5725,34 +5879,34 @@
     </row>
     <row r="35" spans="2:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="45"/>
-      <c r="C35" s="94" t="s">
+      <c r="C35" s="110" t="s">
         <v>5</v>
       </c>
-      <c r="D35" s="156"/>
-      <c r="E35" s="95"/>
+      <c r="D35" s="126"/>
+      <c r="E35" s="111"/>
       <c r="F35" s="34" t="s">
         <v>131</v>
       </c>
       <c r="G35" s="32"/>
-      <c r="H35" s="94" t="s">
+      <c r="H35" s="110" t="s">
         <v>99</v>
       </c>
-      <c r="I35" s="95"/>
+      <c r="I35" s="111"/>
       <c r="J35" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="K35" s="94" t="s">
+      <c r="K35" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="L35" s="95"/>
+      <c r="L35" s="111"/>
       <c r="M35" s="34" t="s">
         <v>131</v>
       </c>
       <c r="N35" s="32"/>
-      <c r="O35" s="94" t="s">
+      <c r="O35" s="110" t="s">
         <v>100</v>
       </c>
-      <c r="P35" s="95"/>
+      <c r="P35" s="111"/>
       <c r="Q35" s="34" t="s">
         <v>131</v>
       </c>
@@ -5798,23 +5952,23 @@
     </row>
     <row r="38" spans="2:18" s="68" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="66"/>
-      <c r="C38" s="157" t="s">
+      <c r="C38" s="121" t="s">
         <v>105</v>
       </c>
-      <c r="D38" s="157"/>
-      <c r="E38" s="157"/>
-      <c r="F38" s="157"/>
-      <c r="G38" s="157"/>
-      <c r="H38" s="157"/>
-      <c r="I38" s="157"/>
-      <c r="J38" s="157"/>
-      <c r="K38" s="157"/>
-      <c r="L38" s="157"/>
-      <c r="M38" s="157"/>
-      <c r="N38" s="157"/>
-      <c r="O38" s="157"/>
-      <c r="P38" s="157"/>
-      <c r="Q38" s="157"/>
+      <c r="D38" s="121"/>
+      <c r="E38" s="121"/>
+      <c r="F38" s="121"/>
+      <c r="G38" s="121"/>
+      <c r="H38" s="121"/>
+      <c r="I38" s="121"/>
+      <c r="J38" s="121"/>
+      <c r="K38" s="121"/>
+      <c r="L38" s="121"/>
+      <c r="M38" s="121"/>
+      <c r="N38" s="121"/>
+      <c r="O38" s="121"/>
+      <c r="P38" s="121"/>
+      <c r="Q38" s="121"/>
       <c r="R38" s="67"/>
     </row>
     <row r="39" spans="2:18" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5831,102 +5985,102 @@
     </row>
     <row r="41" spans="2:18" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="45"/>
-      <c r="C41" s="78" t="s">
+      <c r="C41" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="D41" s="78" t="s">
+      <c r="D41" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="E41" s="78" t="s">
+      <c r="E41" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="F41" s="101" t="s">
+      <c r="F41" s="112" t="s">
         <v>0</v>
       </c>
-      <c r="G41" s="143"/>
-      <c r="H41" s="143"/>
-      <c r="I41" s="102"/>
-      <c r="J41" s="78" t="s">
+      <c r="G41" s="122"/>
+      <c r="H41" s="122"/>
+      <c r="I41" s="113"/>
+      <c r="J41" s="74" t="s">
         <v>101</v>
       </c>
-      <c r="K41" s="93" t="s">
+      <c r="K41" s="107" t="s">
         <v>1</v>
       </c>
-      <c r="L41" s="93"/>
-      <c r="M41" s="78" t="s">
+      <c r="L41" s="107"/>
+      <c r="M41" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="N41" s="78" t="s">
+      <c r="N41" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="O41" s="78" t="s">
+      <c r="O41" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="P41" s="93" t="s">
+      <c r="P41" s="107" t="s">
         <v>100</v>
       </c>
-      <c r="Q41" s="93"/>
+      <c r="Q41" s="107"/>
       <c r="R41" s="46"/>
     </row>
     <row r="42" spans="2:18" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="45"/>
-      <c r="C42" s="69">
+      <c r="C42" s="156">
         <v>1</v>
       </c>
-      <c r="D42" s="69">
-        <v>8</v>
-      </c>
-      <c r="E42" s="70">
+      <c r="D42" s="156">
+        <v>4</v>
+      </c>
+      <c r="E42" s="156">
         <v>22210</v>
       </c>
-      <c r="F42" s="140" t="s">
-        <v>149</v>
-      </c>
-      <c r="G42" s="141"/>
-      <c r="H42" s="141"/>
-      <c r="I42" s="142"/>
-      <c r="J42" s="71" t="s">
-        <v>150</v>
-      </c>
-      <c r="K42" s="127">
-        <v>113</v>
-      </c>
-      <c r="L42" s="128"/>
-      <c r="M42" s="72">
+      <c r="F42" s="157" t="s">
+        <v>160</v>
+      </c>
+      <c r="G42" s="158"/>
+      <c r="H42" s="158"/>
+      <c r="I42" s="159"/>
+      <c r="J42" s="160" t="s">
+        <v>146</v>
+      </c>
+      <c r="K42" s="161">
+        <v>39</v>
+      </c>
+      <c r="L42" s="162"/>
+      <c r="M42" s="163">
         <v>371</v>
       </c>
-      <c r="N42" s="72">
+      <c r="N42" s="163">
         <f>K42*M42</f>
-        <v>41923</v>
-      </c>
-      <c r="O42" s="69" t="s">
-        <v>151</v>
-      </c>
-      <c r="P42" s="140" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q42" s="142"/>
+        <v>14469</v>
+      </c>
+      <c r="O42" s="156" t="s">
+        <v>162</v>
+      </c>
+      <c r="P42" s="157" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q42" s="159"/>
       <c r="R42" s="46"/>
     </row>
     <row r="43" spans="2:18" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="45"/>
-      <c r="C43" s="73">
+      <c r="C43" s="69">
         <v>2</v>
       </c>
-      <c r="D43" s="73"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="136"/>
-      <c r="G43" s="137"/>
-      <c r="H43" s="137"/>
-      <c r="I43" s="138"/>
-      <c r="J43" s="75"/>
-      <c r="K43" s="75"/>
-      <c r="L43" s="76"/>
-      <c r="M43" s="77"/>
-      <c r="N43" s="77"/>
-      <c r="O43" s="73"/>
-      <c r="P43" s="125"/>
-      <c r="Q43" s="126"/>
+      <c r="D43" s="69"/>
+      <c r="E43" s="70"/>
+      <c r="F43" s="123"/>
+      <c r="G43" s="124"/>
+      <c r="H43" s="124"/>
+      <c r="I43" s="125"/>
+      <c r="J43" s="71"/>
+      <c r="K43" s="71"/>
+      <c r="L43" s="72"/>
+      <c r="M43" s="73"/>
+      <c r="N43" s="73"/>
+      <c r="O43" s="69"/>
+      <c r="P43" s="127"/>
+      <c r="Q43" s="128"/>
       <c r="R43" s="46"/>
     </row>
     <row r="44" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5937,13 +6091,13 @@
       </c>
       <c r="N44" s="40">
         <f>SUM(N42:N43)</f>
-        <v>41923</v>
-      </c>
-      <c r="O44" s="144" t="s">
+        <v>14469</v>
+      </c>
+      <c r="O44" s="146" t="s">
         <v>123</v>
       </c>
-      <c r="P44" s="145"/>
-      <c r="Q44" s="145"/>
+      <c r="P44" s="147"/>
+      <c r="Q44" s="147"/>
       <c r="R44" s="46"/>
     </row>
     <row r="45" spans="2:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5956,163 +6110,163 @@
     </row>
     <row r="46" spans="2:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="45"/>
-      <c r="C46" s="78" t="s">
+      <c r="C46" s="74" t="s">
         <v>118</v>
       </c>
-      <c r="D46" s="78" t="s">
+      <c r="D46" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="E46" s="78" t="s">
+      <c r="E46" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="F46" s="101" t="s">
+      <c r="F46" s="112" t="s">
         <v>0</v>
       </c>
-      <c r="G46" s="143"/>
-      <c r="H46" s="143"/>
-      <c r="I46" s="102"/>
-      <c r="J46" s="78" t="s">
+      <c r="G46" s="122"/>
+      <c r="H46" s="122"/>
+      <c r="I46" s="113"/>
+      <c r="J46" s="74" t="s">
         <v>101</v>
       </c>
-      <c r="K46" s="93" t="s">
+      <c r="K46" s="107" t="s">
         <v>1</v>
       </c>
-      <c r="L46" s="93"/>
-      <c r="M46" s="78" t="s">
+      <c r="L46" s="107"/>
+      <c r="M46" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="N46" s="78" t="s">
+      <c r="N46" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="O46" s="78" t="s">
+      <c r="O46" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="P46" s="93" t="s">
+      <c r="P46" s="107" t="s">
         <v>100</v>
       </c>
-      <c r="Q46" s="93"/>
+      <c r="Q46" s="107"/>
       <c r="R46" s="46"/>
     </row>
     <row r="47" spans="2:18" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="45"/>
-      <c r="C47" s="69">
+      <c r="C47" s="156">
         <v>1</v>
       </c>
-      <c r="D47" s="69">
-        <v>8</v>
-      </c>
-      <c r="E47" s="70">
+      <c r="D47" s="156">
+        <v>4</v>
+      </c>
+      <c r="E47" s="156">
         <v>22210</v>
       </c>
-      <c r="F47" s="140" t="s">
-        <v>153</v>
-      </c>
-      <c r="G47" s="141"/>
-      <c r="H47" s="141"/>
-      <c r="I47" s="142"/>
-      <c r="J47" s="71" t="s">
-        <v>150</v>
-      </c>
-      <c r="K47" s="127">
-        <v>1</v>
-      </c>
-      <c r="L47" s="128"/>
-      <c r="M47" s="72">
+      <c r="F47" s="157" t="s">
+        <v>161</v>
+      </c>
+      <c r="G47" s="158"/>
+      <c r="H47" s="158"/>
+      <c r="I47" s="159"/>
+      <c r="J47" s="160" t="s">
+        <v>146</v>
+      </c>
+      <c r="K47" s="161">
+        <v>38</v>
+      </c>
+      <c r="L47" s="162"/>
+      <c r="M47" s="163">
         <v>371</v>
       </c>
-      <c r="N47" s="72">
+      <c r="N47" s="163">
         <f>K47*M47</f>
-        <v>371</v>
-      </c>
-      <c r="O47" s="69" t="s">
-        <v>154</v>
-      </c>
-      <c r="P47" s="140" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q47" s="142"/>
+        <v>14098</v>
+      </c>
+      <c r="O47" s="156" t="s">
+        <v>147</v>
+      </c>
+      <c r="P47" s="157" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q47" s="159"/>
       <c r="R47" s="46"/>
     </row>
     <row r="48" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="45"/>
-      <c r="C48" s="73">
+      <c r="C48" s="164">
         <v>2</v>
       </c>
-      <c r="D48" s="73">
-        <v>8</v>
-      </c>
-      <c r="E48" s="70">
+      <c r="D48" s="164">
+        <v>4</v>
+      </c>
+      <c r="E48" s="152">
         <v>22210</v>
       </c>
-      <c r="F48" s="136" t="s">
-        <v>149</v>
-      </c>
-      <c r="G48" s="137"/>
-      <c r="H48" s="137"/>
-      <c r="I48" s="138"/>
-      <c r="J48" s="75" t="s">
-        <v>150</v>
-      </c>
-      <c r="K48" s="125">
-        <v>112</v>
-      </c>
-      <c r="L48" s="126"/>
-      <c r="M48" s="77">
+      <c r="F48" s="165" t="s">
+        <v>165</v>
+      </c>
+      <c r="G48" s="166"/>
+      <c r="H48" s="166"/>
+      <c r="I48" s="167"/>
+      <c r="J48" s="168" t="s">
+        <v>146</v>
+      </c>
+      <c r="K48" s="169">
+        <v>1</v>
+      </c>
+      <c r="L48" s="170"/>
+      <c r="M48" s="171">
         <v>371</v>
       </c>
-      <c r="N48" s="72">
+      <c r="N48" s="155">
         <f>K48*M48</f>
-        <v>41552</v>
-      </c>
-      <c r="O48" s="73" t="s">
-        <v>151</v>
-      </c>
-      <c r="P48" s="140" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q48" s="142"/>
+        <v>371</v>
+      </c>
+      <c r="O48" s="164" t="s">
+        <v>148</v>
+      </c>
+      <c r="P48" s="153" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q48" s="154"/>
       <c r="R48" s="46"/>
     </row>
     <row r="49" spans="2:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="45"/>
-      <c r="C49" s="73">
+      <c r="C49" s="69">
         <v>3</v>
       </c>
-      <c r="D49" s="73"/>
-      <c r="E49" s="74"/>
-      <c r="F49" s="136"/>
-      <c r="G49" s="137"/>
-      <c r="H49" s="137"/>
-      <c r="I49" s="138"/>
-      <c r="J49" s="75"/>
-      <c r="K49" s="125"/>
-      <c r="L49" s="126"/>
-      <c r="M49" s="77"/>
-      <c r="N49" s="77"/>
-      <c r="O49" s="73"/>
-      <c r="P49" s="136"/>
-      <c r="Q49" s="138"/>
+      <c r="D49" s="69"/>
+      <c r="E49" s="70"/>
+      <c r="F49" s="123"/>
+      <c r="G49" s="124"/>
+      <c r="H49" s="124"/>
+      <c r="I49" s="125"/>
+      <c r="J49" s="71"/>
+      <c r="K49" s="127"/>
+      <c r="L49" s="128"/>
+      <c r="M49" s="73"/>
+      <c r="N49" s="73"/>
+      <c r="O49" s="69"/>
+      <c r="P49" s="123"/>
+      <c r="Q49" s="125"/>
       <c r="R49" s="46"/>
     </row>
     <row r="50" spans="2:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="45"/>
-      <c r="C50" s="73">
+      <c r="C50" s="69">
         <v>4</v>
       </c>
-      <c r="D50" s="73"/>
-      <c r="E50" s="74"/>
-      <c r="F50" s="136"/>
-      <c r="G50" s="137"/>
-      <c r="H50" s="137"/>
-      <c r="I50" s="138"/>
-      <c r="J50" s="75"/>
-      <c r="K50" s="125"/>
-      <c r="L50" s="126"/>
-      <c r="M50" s="77"/>
-      <c r="N50" s="77"/>
-      <c r="O50" s="73"/>
-      <c r="P50" s="136"/>
-      <c r="Q50" s="138"/>
+      <c r="D50" s="69"/>
+      <c r="E50" s="70"/>
+      <c r="F50" s="123"/>
+      <c r="G50" s="124"/>
+      <c r="H50" s="124"/>
+      <c r="I50" s="125"/>
+      <c r="J50" s="71"/>
+      <c r="K50" s="127"/>
+      <c r="L50" s="128"/>
+      <c r="M50" s="73"/>
+      <c r="N50" s="73"/>
+      <c r="O50" s="69"/>
+      <c r="P50" s="123"/>
+      <c r="Q50" s="125"/>
       <c r="R50" s="46"/>
     </row>
     <row r="51" spans="2:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6122,13 +6276,13 @@
       </c>
       <c r="N51" s="40">
         <f>SUM(N47:N50)</f>
-        <v>41923</v>
-      </c>
-      <c r="O51" s="139" t="s">
+        <v>14469</v>
+      </c>
+      <c r="O51" s="145" t="s">
         <v>124</v>
       </c>
-      <c r="P51" s="139"/>
-      <c r="Q51" s="139"/>
+      <c r="P51" s="145"/>
+      <c r="Q51" s="145"/>
       <c r="R51" s="46"/>
     </row>
     <row r="52" spans="2:18" ht="6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6150,23 +6304,23 @@
     </row>
     <row r="54" spans="2:18" s="63" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="61"/>
-      <c r="C54" s="90" t="s">
+      <c r="C54" s="98" t="s">
         <v>106</v>
       </c>
-      <c r="D54" s="90"/>
-      <c r="E54" s="90"/>
-      <c r="F54" s="90"/>
-      <c r="G54" s="90"/>
-      <c r="H54" s="90"/>
-      <c r="I54" s="90"/>
-      <c r="J54" s="90"/>
-      <c r="K54" s="90"/>
-      <c r="L54" s="90"/>
-      <c r="M54" s="90"/>
-      <c r="N54" s="90"/>
-      <c r="O54" s="90"/>
-      <c r="P54" s="90"/>
-      <c r="Q54" s="90"/>
+      <c r="D54" s="98"/>
+      <c r="E54" s="98"/>
+      <c r="F54" s="98"/>
+      <c r="G54" s="98"/>
+      <c r="H54" s="98"/>
+      <c r="I54" s="98"/>
+      <c r="J54" s="98"/>
+      <c r="K54" s="98"/>
+      <c r="L54" s="98"/>
+      <c r="M54" s="98"/>
+      <c r="N54" s="98"/>
+      <c r="O54" s="98"/>
+      <c r="P54" s="98"/>
+      <c r="Q54" s="98"/>
       <c r="R54" s="65"/>
     </row>
     <row r="55" spans="2:18" ht="3" customHeight="1" x14ac:dyDescent="0.25">
@@ -6186,21 +6340,21 @@
     </row>
     <row r="58" spans="2:18" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="45"/>
-      <c r="C58" s="113"/>
-      <c r="D58" s="113"/>
-      <c r="E58" s="113"/>
-      <c r="F58" s="113"/>
-      <c r="G58" s="113"/>
-      <c r="H58" s="113"/>
-      <c r="I58" s="113"/>
-      <c r="J58" s="113"/>
-      <c r="K58" s="113"/>
-      <c r="L58" s="113"/>
-      <c r="M58" s="113"/>
-      <c r="N58" s="113"/>
-      <c r="O58" s="113"/>
-      <c r="P58" s="113"/>
-      <c r="Q58" s="113"/>
+      <c r="C58" s="108"/>
+      <c r="D58" s="108"/>
+      <c r="E58" s="108"/>
+      <c r="F58" s="108"/>
+      <c r="G58" s="108"/>
+      <c r="H58" s="108"/>
+      <c r="I58" s="108"/>
+      <c r="J58" s="108"/>
+      <c r="K58" s="108"/>
+      <c r="L58" s="108"/>
+      <c r="M58" s="108"/>
+      <c r="N58" s="108"/>
+      <c r="O58" s="108"/>
+      <c r="P58" s="108"/>
+      <c r="Q58" s="108"/>
       <c r="R58" s="46"/>
     </row>
     <row r="59" spans="2:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6224,22 +6378,33 @@
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="P47:Q47"/>
-    <mergeCell ref="P41:Q41"/>
-    <mergeCell ref="C38:Q38"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="O35:P35"/>
-    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="C23:Q23"/>
+    <mergeCell ref="C27:Q27"/>
+    <mergeCell ref="C29:Q29"/>
+    <mergeCell ref="C28:Q28"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="H17:Q17"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="H19:Q19"/>
+    <mergeCell ref="H21:Q21"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="C31:Q31"/>
+    <mergeCell ref="P46:Q46"/>
+    <mergeCell ref="C58:G58"/>
+    <mergeCell ref="H58:L58"/>
+    <mergeCell ref="M58:Q58"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="C54:Q54"/>
+    <mergeCell ref="O51:Q51"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="P49:Q49"/>
+    <mergeCell ref="P50:Q50"/>
+    <mergeCell ref="F50:I50"/>
     <mergeCell ref="K48:L48"/>
     <mergeCell ref="C3:Q3"/>
     <mergeCell ref="H25:K25"/>
@@ -6256,38 +6421,27 @@
     <mergeCell ref="H15:Q15"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="P48:Q48"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="O35:P35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="P47:Q47"/>
+    <mergeCell ref="P41:Q41"/>
+    <mergeCell ref="C38:Q38"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F43:I43"/>
     <mergeCell ref="K46:L46"/>
     <mergeCell ref="K42:L42"/>
-    <mergeCell ref="C58:G58"/>
-    <mergeCell ref="H58:L58"/>
-    <mergeCell ref="M58:Q58"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="C54:Q54"/>
-    <mergeCell ref="O51:Q51"/>
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="P49:Q49"/>
-    <mergeCell ref="P50:Q50"/>
     <mergeCell ref="F47:I47"/>
     <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F50:I50"/>
     <mergeCell ref="O44:Q44"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="P43:Q43"/>
-    <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="C31:Q31"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="H17:Q17"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="H19:Q19"/>
-    <mergeCell ref="H21:Q21"/>
-    <mergeCell ref="C23:Q23"/>
-    <mergeCell ref="C27:Q27"/>
-    <mergeCell ref="C29:Q29"/>
-    <mergeCell ref="C28:Q28"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="P46:Q46"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H32:I32 H26:I26" xr:uid="{00000000-0002-0000-0200-000000000000}">

</xml_diff>